<commit_message>
feat(navigation): rename Occupancy to Campaign Tracker and Campaign Tracker to Latest Booking
</commit_message>
<xml_diff>
--- a/client/dist/sample_campaign_tracker_import.xlsx
+++ b/client/dist/sample_campaign_tracker_import.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Campaign Tracker" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Latest Booking" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Instructions &amp; Guide" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="87">
   <si>
-    <t>MEDIA BUZZ — CAMPAIGN TRACKER IMPORT TEMPLATE</t>
+    <t>MEDIA BUZZ — LATEST BOOKING IMPORT TEMPLATE</t>
   </si>
   <si>
     <t>Site Code</t>
@@ -167,7 +167,7 @@
     <t>61x10 ft</t>
   </si>
   <si>
-    <t>CAMPAIGN TRACKER IMPORT FIELD SPECIFICATION GUIDE</t>
+    <t>LATEST BOOKING IMPORT FIELD SPECIFICATION GUIDE</t>
   </si>
   <si>
     <t>Column Header</t>

</xml_diff>